<commit_message>
Add custom weighting and starting continent controls
</commit_message>
<xml_diff>
--- a/assets/data/generatordata.xlsx
+++ b/assets/data/generatordata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mthak\Desktop\pf2e-generator\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACE15F5-FCB4-4AA2-84CC-29EEB3B1E559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62554153-024D-4358-878F-084062FEB87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{12225E00-D84F-438D-9971-6445E1072934}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{12225E00-D84F-438D-9971-6445E1072934}"/>
   </bookViews>
   <sheets>
     <sheet name="Ancestries" sheetId="2" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9156" uniqueCount="2158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9210" uniqueCount="2166">
   <si>
     <t>ancestry</t>
   </si>
@@ -6522,6 +6522,30 @@
   </si>
   <si>
     <t>specific_weapon</t>
+  </si>
+  <si>
+    <t>rarity_garund</t>
+  </si>
+  <si>
+    <t>rarity_tianxia</t>
+  </si>
+  <si>
+    <t>rarity_avistan</t>
+  </si>
+  <si>
+    <t>Iblydos</t>
+  </si>
+  <si>
+    <t>Kelesh</t>
+  </si>
+  <si>
+    <t>Vudra</t>
+  </si>
+  <si>
+    <t>rarity_casmaron</t>
+  </si>
+  <si>
+    <t>rarity_arcadia</t>
   </si>
 </sst>
 </file>
@@ -6558,7 +6582,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -6581,11 +6605,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -6604,6 +6639,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6939,15 +6977,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3D1795-EDE3-4633-8891-F0CE552D71CB}">
-  <dimension ref="A1:D51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr defaultColWidth="102.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -6955,13 +6997,28 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2160</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2158</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2159</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2165</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>2164</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>34</v>
       </c>
@@ -6969,11 +7026,16 @@
         <v>7</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>46</v>
       </c>
@@ -6981,11 +7043,16 @@
         <v>7</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>54</v>
       </c>
@@ -6994,10 +7061,17 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>62</v>
       </c>
@@ -7006,10 +7080,17 @@
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>71</v>
       </c>
@@ -7017,11 +7098,16 @@
         <v>7</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>79</v>
       </c>
@@ -7029,11 +7115,16 @@
         <v>7</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>83</v>
       </c>
@@ -7041,11 +7132,16 @@
         <v>7</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>97</v>
       </c>
@@ -7053,23 +7149,39 @@
         <v>7</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>105</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2" t="s">
+      <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>111</v>
       </c>
@@ -7077,11 +7189,20 @@
         <v>11</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="2"/>
+      <c r="E11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>122</v>
       </c>
@@ -7090,10 +7211,23 @@
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>130</v>
       </c>
@@ -7102,10 +7236,21 @@
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>137</v>
       </c>
@@ -7114,10 +7259,21 @@
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>141</v>
       </c>
@@ -7126,10 +7282,19 @@
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>149</v>
       </c>
@@ -7138,10 +7303,21 @@
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>156</v>
       </c>
@@ -7149,11 +7325,18 @@
         <v>11</v>
       </c>
       <c r="C17" s="2"/>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="2"/>
+      <c r="E17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>163</v>
       </c>
@@ -7162,10 +7345,17 @@
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>174</v>
       </c>
@@ -7174,10 +7364,17 @@
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>184</v>
       </c>
@@ -7185,11 +7382,16 @@
         <v>11</v>
       </c>
       <c r="C20" s="2"/>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>190</v>
       </c>
@@ -7197,23 +7399,39 @@
         <v>11</v>
       </c>
       <c r="C21" s="2"/>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>197</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="D22" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>205</v>
       </c>
@@ -7221,35 +7439,64 @@
         <v>11</v>
       </c>
       <c r="C23" s="2"/>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="2"/>
+      <c r="E23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>210</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="D24" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>216</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="D25" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>222</v>
       </c>
@@ -7257,11 +7504,18 @@
         <v>11</v>
       </c>
       <c r="C26" s="2"/>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="2"/>
+      <c r="E26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>229</v>
       </c>
@@ -7270,34 +7524,61 @@
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>236</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2" t="s">
+      <c r="C28" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>241</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="D29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>247</v>
       </c>
@@ -7305,11 +7586,16 @@
         <v>31</v>
       </c>
       <c r="C30" s="2"/>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>254</v>
       </c>
@@ -7317,11 +7603,16 @@
         <v>31</v>
       </c>
       <c r="C31" s="2"/>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>260</v>
       </c>
@@ -7329,11 +7620,16 @@
         <v>31</v>
       </c>
       <c r="C32" s="2"/>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>265</v>
       </c>
@@ -7341,11 +7637,16 @@
         <v>31</v>
       </c>
       <c r="C33" s="2"/>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>270</v>
       </c>
@@ -7353,11 +7654,16 @@
         <v>31</v>
       </c>
       <c r="C34" s="2"/>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>276</v>
       </c>
@@ -7365,11 +7671,16 @@
         <v>31</v>
       </c>
       <c r="C35" s="2"/>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>283</v>
       </c>
@@ -7377,11 +7688,16 @@
         <v>31</v>
       </c>
       <c r="C36" s="2"/>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>291</v>
       </c>
@@ -7389,11 +7705,16 @@
         <v>31</v>
       </c>
       <c r="C37" s="2"/>
-      <c r="D37" s="2" t="s">
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>296</v>
       </c>
@@ -7401,11 +7722,16 @@
         <v>31</v>
       </c>
       <c r="C38" s="2"/>
-      <c r="D38" s="2" t="s">
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>302</v>
       </c>
@@ -7413,11 +7739,16 @@
         <v>31</v>
       </c>
       <c r="C39" s="2"/>
-      <c r="D39" s="2" t="s">
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>308</v>
       </c>
@@ -7425,11 +7756,18 @@
         <v>31</v>
       </c>
       <c r="C40" s="2"/>
-      <c r="D40" s="2" t="s">
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>314</v>
       </c>
@@ -7437,11 +7775,16 @@
         <v>31</v>
       </c>
       <c r="C41" s="2"/>
-      <c r="D41" s="2" t="s">
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>322</v>
       </c>
@@ -7449,11 +7792,16 @@
         <v>31</v>
       </c>
       <c r="C42" s="2"/>
-      <c r="D42" s="2" t="s">
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>328</v>
       </c>
@@ -7462,24 +7810,36 @@
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>334</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="I44" s="2" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>340</v>
       </c>
@@ -7487,11 +7847,16 @@
         <v>31</v>
       </c>
       <c r="C45" s="2"/>
-      <c r="D45" s="2" t="s">
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>348</v>
       </c>
@@ -7499,11 +7864,16 @@
         <v>31</v>
       </c>
       <c r="C46" s="2"/>
-      <c r="D46" s="2" t="s">
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>359</v>
       </c>
@@ -7511,11 +7881,16 @@
         <v>31</v>
       </c>
       <c r="C47" s="2"/>
-      <c r="D47" s="2" t="s">
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>365</v>
       </c>
@@ -7523,11 +7898,16 @@
         <v>31</v>
       </c>
       <c r="C48" s="2"/>
-      <c r="D48" s="2" t="s">
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>370</v>
       </c>
@@ -7535,11 +7915,18 @@
         <v>31</v>
       </c>
       <c r="C49" s="2"/>
-      <c r="D49" s="2" t="s">
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>377</v>
       </c>
@@ -7547,11 +7934,16 @@
         <v>31</v>
       </c>
       <c r="C50" s="2"/>
-      <c r="D50" s="2" t="s">
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>384</v>
       </c>
@@ -7559,7 +7951,12 @@
         <v>31</v>
       </c>
       <c r="C51" s="2"/>
-      <c r="D51" s="2" t="s">
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -31044,7 +31441,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AF39BE0-A267-465D-94EE-F339AD54ABEF}">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultColWidth="64.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
@@ -31776,12 +32173,28 @@
     </row>
     <row r="81" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>1288</v>
+        <v>2161</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>1288</v>
       </c>
       <c r="C81" s="2"/>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="7" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B82" s="7" t="s">
+        <v>1288</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="7" t="s">
+        <v>2163</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>1288</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>